<commit_message>
Widen template spreadsheet columns to fit content
Set an explicit width for every column in both Excel templates
(Players.xlsx and classification-results-spreadsheet-template.xlsx),
sized to the longest content (header or cell) plus a small margin, so no
information is cut off when the templates are opened.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/assessment_forms/assets/Players.xlsx
+++ b/tools/assessment_forms/assets/Players.xlsx
@@ -420,11 +420,13 @@
   <dimension ref="A1:G100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11.38" customWidth="1" min="1" max="1"/>
-    <col width="31.38" customWidth="1" min="2" max="2"/>
-    <col width="18.88" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="50.13" customWidth="1" min="7" max="7"/>
+    <col width="8.5" customWidth="1" min="1" max="1"/>
+    <col width="15.5" customWidth="1" min="2" max="2"/>
+    <col width="16.5" customWidth="1" min="3" max="3"/>
+    <col width="8.5" customWidth="1" min="4" max="4"/>
+    <col width="12.5" customWidth="1" min="5" max="5"/>
+    <col width="12.5" customWidth="1" min="6" max="6"/>
+    <col width="24.5" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1397,11 +1399,13 @@
   <dimension ref="A1:G100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11.38" customWidth="1" min="1" max="1"/>
-    <col width="31.38" customWidth="1" min="2" max="2"/>
-    <col width="18.88" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="50.13" customWidth="1" min="7" max="7"/>
+    <col width="8.5" customWidth="1" min="1" max="1"/>
+    <col width="15.5" customWidth="1" min="2" max="2"/>
+    <col width="16.5" customWidth="1" min="3" max="3"/>
+    <col width="8.5" customWidth="1" min="4" max="4"/>
+    <col width="12.5" customWidth="1" min="5" max="5"/>
+    <col width="12.5" customWidth="1" min="6" max="6"/>
+    <col width="24.5" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2374,11 +2378,13 @@
   <dimension ref="A1:G100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11.38" customWidth="1" min="1" max="1"/>
-    <col width="31.38" customWidth="1" min="2" max="2"/>
-    <col width="18.88" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="50.13" customWidth="1" min="7" max="7"/>
+    <col width="8.5" customWidth="1" min="1" max="1"/>
+    <col width="15.5" customWidth="1" min="2" max="2"/>
+    <col width="16.5" customWidth="1" min="3" max="3"/>
+    <col width="8.5" customWidth="1" min="4" max="4"/>
+    <col width="12.5" customWidth="1" min="5" max="5"/>
+    <col width="12.5" customWidth="1" min="6" max="6"/>
+    <col width="24.5" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3351,11 +3357,13 @@
   <dimension ref="A1:G100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11.38" customWidth="1" min="1" max="1"/>
-    <col width="31.38" customWidth="1" min="2" max="2"/>
-    <col width="18.88" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="50.13" customWidth="1" min="7" max="7"/>
+    <col width="8.5" customWidth="1" min="1" max="1"/>
+    <col width="15.5" customWidth="1" min="2" max="2"/>
+    <col width="16.5" customWidth="1" min="3" max="3"/>
+    <col width="8.5" customWidth="1" min="4" max="4"/>
+    <col width="12.5" customWidth="1" min="5" max="5"/>
+    <col width="12.5" customWidth="1" min="6" max="6"/>
+    <col width="24.5" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>